<commit_message>
modified modules to run new FAO GAEZ updated data
</commit_message>
<xml_diff>
--- a/data/crops/crop_residue_data.xlsx
+++ b/data/crops/crop_residue_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{9BD4F013-961F-47EC-97FA-9734F9CC6039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BD420D6E-47E9-4E85-A249-DE3352C786F9}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{9BD4F013-961F-47EC-97FA-9734F9CC6039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F5FC189B-C5FD-5280-B794-7013C4C8685A}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{2E930A77-F482-4EC5-8F8A-15553659F0D1}"/>
   </bookViews>

</xml_diff>